<commit_message>
component list updated, all footprints updated and now they are compatible to produce with hand (no 0402 size)
</commit_message>
<xml_diff>
--- a/ESC_Component_List.xlsx
+++ b/ESC_Component_List.xlsx
@@ -5,22 +5,22 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alper\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alper\Desktop\UNİ_DERS\bitirme_projesi\New folder\BLDC-Motor-Driver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F8B30A-7056-47A0-82F1-6BD57EC3CE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A3D51A-93C2-4B0D-9FF0-01C2B1DFC266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t>Digi-Key: Shopping Cart</t>
   </si>
@@ -118,15 +118,6 @@
     <t>DIODE SCHOTTKY 80V 1A DO214AC</t>
   </si>
   <si>
-    <t>CSNL2512FT3L00CT-ND</t>
-  </si>
-  <si>
-    <t>CSNL2512FT3L00</t>
-  </si>
-  <si>
-    <t>RES 0.003 OHM 1% 3W 2512</t>
-  </si>
-  <si>
     <t>RMCF0603ZT0R00CT-ND</t>
   </si>
   <si>
@@ -305,13 +296,76 @@
   </si>
   <si>
     <t>IC TRANSCEIVER 1/1 8SOIC</t>
+  </si>
+  <si>
+    <t>P12011CT-ND</t>
+  </si>
+  <si>
+    <t>ERT-J1VG103FA</t>
+  </si>
+  <si>
+    <t>THERMISTOR NTC 10KOHM 3380K 0603</t>
+  </si>
+  <si>
+    <t>CRF2512-FZ-R002ELFCT-ND</t>
+  </si>
+  <si>
+    <t>CRF2512-FZ-R002ELF</t>
+  </si>
+  <si>
+    <t>RES 0.002 OHM 1% 2W 2512</t>
+  </si>
+  <si>
+    <t>311-5.6KDCT-ND</t>
+  </si>
+  <si>
+    <t>RT0603DRD075K6L</t>
+  </si>
+  <si>
+    <t>RES SMD 5.6K OHM 0.5% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>MMSZ3V3T1GOSCT-ND</t>
+  </si>
+  <si>
+    <t>MMSZ3V3T1G</t>
+  </si>
+  <si>
+    <t>DIODE ZENER 3.3V 500MW SOD123</t>
+  </si>
+  <si>
+    <t>2223-TS04-66-73-BK-260-SMT-ND</t>
+  </si>
+  <si>
+    <t>TS04-66-73-BK-260-SMT</t>
+  </si>
+  <si>
+    <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
+  </si>
+  <si>
+    <t>732-7817-1-ND</t>
+  </si>
+  <si>
+    <t>CAP CER 33PF 16V C0G/NP0 0805</t>
+  </si>
+  <si>
+    <t>https://www.direnc.net/1uf-16v-10-x5r-603-smd-kondansator</t>
+  </si>
+  <si>
+    <t>1uF 6.3V 10% x5R 603 SMD Kondansatör</t>
+  </si>
+  <si>
+    <t>1uF 16V 10% x5R 603 SMD Kondansatör</t>
+  </si>
+  <si>
+    <t>  100nF 50V 10% x7R 805 SMD Kondansatör</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -319,6 +373,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -339,10 +399,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -351,8 +412,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -665,12 +728,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
-    <col min="3" max="3" width="36.42578125" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" customWidth="1"/>
     <col min="4" max="4" width="32.42578125" customWidth="1"/>
     <col min="5" max="5" width="43.140625" customWidth="1"/>
     <col min="6" max="6" width="24.28515625" customWidth="1"/>
@@ -846,7 +909,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
         <v>23</v>
@@ -858,7 +921,7 @@
         <v>25</v>
       </c>
       <c r="G7" s="2">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2">
         <v>0</v>
@@ -867,7 +930,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
       <c r="J7" s="3">
-        <v>0.11</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -951,10 +1014,10 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>0.495</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="J10" s="3">
-        <v>4.95</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -980,10 +1043,10 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>6.0000000000000001E-3</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="J11" s="3">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1009,10 +1072,10 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>1.0999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="J12" s="3">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -1020,7 +1083,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1032,16 +1095,16 @@
         <v>43</v>
       </c>
       <c r="G13" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H13" s="2">
         <v>0</v>
       </c>
       <c r="I13">
-        <v>0.01</v>
+        <v>0.26</v>
       </c>
       <c r="J13" s="3">
-        <v>0.1</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1049,7 +1112,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1061,16 +1124,16 @@
         <v>46</v>
       </c>
       <c r="G14" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H14" s="2">
         <v>0</v>
       </c>
       <c r="I14">
-        <v>0.26</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="J14" s="3">
-        <v>0.52</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -1078,7 +1141,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -1090,16 +1153,16 @@
         <v>49</v>
       </c>
       <c r="G15" s="2">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H15" s="2">
         <v>0</v>
       </c>
       <c r="I15">
-        <v>4.4999999999999998E-2</v>
+        <v>5.5999999999999999E-3</v>
       </c>
       <c r="J15" s="3">
-        <v>0.45</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1154,10 +1217,10 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>5.5999999999999999E-3</v>
+        <v>1.0800000000000001E-2</v>
       </c>
       <c r="J17" s="3">
-        <v>0.14000000000000001</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -1183,10 +1246,10 @@
         <v>0</v>
       </c>
       <c r="I18">
-        <v>1.0800000000000001E-2</v>
+        <v>8.8000000000000005E-3</v>
       </c>
       <c r="J18" s="3">
-        <v>0.27</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -1194,7 +1257,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1206,16 +1269,16 @@
         <v>61</v>
       </c>
       <c r="G19" s="2">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="H19" s="2">
         <v>0</v>
       </c>
       <c r="I19">
-        <v>8.8000000000000005E-3</v>
+        <v>2.93</v>
       </c>
       <c r="J19" s="3">
-        <v>0.22</v>
+        <v>8.7899999999999991</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -1223,7 +1286,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1235,16 +1298,16 @@
         <v>64</v>
       </c>
       <c r="G20" s="2">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="H20" s="2">
         <v>0</v>
       </c>
       <c r="I20">
-        <v>2.93</v>
+        <v>5.5999999999999999E-3</v>
       </c>
       <c r="J20" s="3">
-        <v>8.7899999999999991</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -1281,7 +1344,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1293,16 +1356,16 @@
         <v>70</v>
       </c>
       <c r="G22" s="2">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H22" s="2">
         <v>0</v>
       </c>
       <c r="I22">
-        <v>5.5999999999999999E-3</v>
+        <v>4.2999999999999997E-2</v>
       </c>
       <c r="J22" s="3">
-        <v>0.14000000000000001</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -1310,7 +1373,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1322,16 +1385,16 @@
         <v>73</v>
       </c>
       <c r="G23" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H23" s="2">
         <v>0</v>
       </c>
       <c r="I23">
-        <v>4.2999999999999997E-2</v>
+        <v>2.09</v>
       </c>
       <c r="J23" s="3">
-        <v>0.43</v>
+        <v>4.18</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -1339,7 +1402,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C24" t="s">
         <v>74</v>
@@ -1351,16 +1414,16 @@
         <v>76</v>
       </c>
       <c r="G24" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H24" s="2">
         <v>0</v>
       </c>
       <c r="I24">
-        <v>2.09</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="J24" s="3">
-        <v>4.18</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -1386,10 +1449,10 @@
         <v>0</v>
       </c>
       <c r="I25">
-        <v>3.2000000000000001E-2</v>
+        <v>0.255</v>
       </c>
       <c r="J25" s="3">
-        <v>0.32</v>
+        <v>2.5499999999999998</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -1397,7 +1460,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1409,16 +1472,16 @@
         <v>82</v>
       </c>
       <c r="G26" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H26" s="2">
         <v>0</v>
       </c>
       <c r="I26">
-        <v>0.255</v>
+        <v>0.33</v>
       </c>
       <c r="J26" s="3">
-        <v>2.5499999999999998</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -1444,10 +1507,10 @@
         <v>0</v>
       </c>
       <c r="I27">
-        <v>0.33</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J27" s="3">
-        <v>0.66</v>
+        <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -1455,7 +1518,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1467,16 +1530,16 @@
         <v>88</v>
       </c>
       <c r="G28" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H28" s="2">
         <v>0</v>
       </c>
       <c r="I28">
-        <v>0.28000000000000003</v>
+        <v>0.15</v>
       </c>
       <c r="J28" s="3">
-        <v>0.56000000000000005</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -1484,7 +1547,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="s">
         <v>89</v>
@@ -1496,16 +1559,16 @@
         <v>91</v>
       </c>
       <c r="G29" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29" s="2">
         <v>0</v>
       </c>
       <c r="I29">
-        <v>0.15</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="J29" s="3">
-        <v>0.15</v>
+        <v>4.4800000000000004</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -1513,7 +1576,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
         <v>92</v>
@@ -1525,22 +1588,219 @@
         <v>94</v>
       </c>
       <c r="G30" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H30" s="2">
         <v>0</v>
       </c>
       <c r="I30">
-        <v>2.2400000000000002</v>
+        <v>0.156</v>
       </c>
       <c r="J30" s="3">
-        <v>4.4800000000000004</v>
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>29</v>
+      </c>
+      <c r="B31" s="2">
+        <v>10</v>
+      </c>
+      <c r="C31" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" t="s">
+        <v>96</v>
+      </c>
+      <c r="E31" t="s">
+        <v>97</v>
+      </c>
+      <c r="G31" s="2">
+        <v>10</v>
+      </c>
+      <c r="H31" s="2">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>0.312</v>
+      </c>
+      <c r="J31" s="3">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>30</v>
+      </c>
+      <c r="B32" s="2">
+        <v>10</v>
+      </c>
+      <c r="C32" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32" t="s">
+        <v>99</v>
+      </c>
+      <c r="E32" t="s">
+        <v>100</v>
+      </c>
+      <c r="G32" s="2">
+        <v>10</v>
+      </c>
+      <c r="H32" s="2">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>0.03</v>
+      </c>
+      <c r="J32" s="3">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>31</v>
+      </c>
+      <c r="B33" s="2">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
+        <v>101</v>
+      </c>
+      <c r="D33" t="s">
+        <v>102</v>
+      </c>
+      <c r="E33" t="s">
+        <v>103</v>
+      </c>
+      <c r="G33" s="2">
+        <v>10</v>
+      </c>
+      <c r="H33" s="2">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="J33" s="3">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>32</v>
+      </c>
+      <c r="B34" s="2">
+        <v>10</v>
+      </c>
+      <c r="C34" t="s">
+        <v>104</v>
+      </c>
+      <c r="D34" t="s">
+        <v>105</v>
+      </c>
+      <c r="E34" t="s">
+        <v>106</v>
+      </c>
+      <c r="G34" s="2">
+        <v>10</v>
+      </c>
+      <c r="H34" s="2">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>0.16</v>
+      </c>
+      <c r="J34" s="3">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>33</v>
+      </c>
+      <c r="B35" s="2">
+        <v>10</v>
+      </c>
+      <c r="C35" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" s="2">
+        <v>885012007013</v>
+      </c>
+      <c r="E35" t="s">
+        <v>108</v>
+      </c>
+      <c r="G35" s="2">
+        <v>10</v>
+      </c>
+      <c r="H35" s="2">
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="J35" s="3">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>34</v>
+      </c>
+      <c r="B36" s="2">
+        <v>20</v>
+      </c>
+      <c r="C36" t="s">
+        <v>110</v>
+      </c>
+      <c r="E36" t="s">
+        <v>109</v>
+      </c>
+      <c r="I36">
+        <f>8/44</f>
+        <v>0.18181818181818182</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>35</v>
+      </c>
+      <c r="B37" s="2">
+        <v>20</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="I37">
+        <f>7/44</f>
+        <v>0.15909090909090909</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>36</v>
+      </c>
+      <c r="B38" s="2">
+        <v>20</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I38">
+        <f>6/44</f>
+        <v>0.13636363636363635</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C37" r:id="rId1" display="https://www.direnc.net/1uf-50v-10-603-smd-kondansator" xr:uid="{13BF0FC5-FB06-4BD5-97C9-9E50FEEDA8C8}"/>
+    <hyperlink ref="C38" r:id="rId2" display="https://www.direnc.net/100nf50v-805-kilif" xr:uid="{E185F8F2-D672-405A-B2DC-0B619D04E544}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>